<commit_message>
docs: complete official assessment submission workbook with all accurate candidate details, observations, fixes, and self-checks
</commit_message>
<xml_diff>
--- a/exports/workbook/IncuBrix_2027_Growth_Engineer_Option_3_AEO_SEO_GEO_Submission_Workbook.xlsx
+++ b/exports/workbook/IncuBrix_2027_Growth_Engineer_Option_3_AEO_SEO_GEO_Submission_Workbook.xlsx
@@ -560,7 +560,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F27"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" style="14" min="1" max="1"/>
     <col width="70" customWidth="1" style="14" min="2" max="2"/>
@@ -617,7 +617,7 @@
       </c>
       <c r="B5" s="23" t="inlineStr">
         <is>
-          <t>GROWTH-ENG-2027-OPT3-001</t>
+          <t>VARNIKA S R</t>
         </is>
       </c>
       <c r="D5" s="24" t="n">
@@ -642,7 +642,7 @@
       </c>
       <c r="B6" s="23" t="inlineStr">
         <is>
-          <t>Growth Engineer Candidate</t>
+          <t>VARNIKA S R</t>
         </is>
       </c>
       <c r="D6" s="24" t="n">
@@ -667,7 +667,7 @@
       </c>
       <c r="B7" s="23" t="inlineStr">
         <is>
-          <t>candidate@incubrix.com</t>
+          <t>srvarnika7@gmail.com</t>
         </is>
       </c>
       <c r="D7" s="24" t="n">
@@ -692,7 +692,7 @@
       </c>
       <c r="B8" s="23" t="inlineStr">
         <is>
-          <t>B.Tech Computer Science &amp; Engineering / AI &amp; Data Science</t>
+          <t>Btech IT</t>
         </is>
       </c>
       <c r="D8" s="24" t="n">
@@ -717,7 +717,7 @@
       </c>
       <c r="B9" s="23" t="inlineStr">
         <is>
-          <t>2026-10-24 09:00 IST</t>
+          <t>24.10.26</t>
         </is>
       </c>
       <c r="D9" s="24" t="n">
@@ -742,7 +742,7 @@
       </c>
       <c r="B10" s="23" t="inlineStr">
         <is>
-          <t>2026-10-31 22:00 IST</t>
+          <t>31.10.26</t>
         </is>
       </c>
       <c r="D10" s="24" t="n">
@@ -767,7 +767,7 @@
       </c>
       <c r="B11" s="23" t="inlineStr">
         <is>
-          <t>submission/</t>
+          <t>https://github.com/Varnika2005/Incubrix2/tree/main/submission</t>
         </is>
       </c>
     </row>
@@ -779,7 +779,7 @@
       </c>
       <c r="B12" s="23" t="inlineStr">
         <is>
-          <t>https://github.com/incubrix/aeo-seo-geo-visibility-engine</t>
+          <t>https://github.com/Varnika2005/Incubrix2.git</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="B13" s="23" t="inlineStr">
         <is>
-          <t>submission/launch_kit/90_DAY_LAUNCH_KIT.md</t>
+          <t>https://github.com/Varnika2005/Incubrix2/blob/main/submission/launch_kit/90_DAY_LAUNCH_KIT.md</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="B14" s="23" t="inlineStr">
         <is>
-          <t>submission/videos/PRODUCT_WALKTHROUGH.mp4</t>
+          <t>https://drive.google.com/drive/folders/1_zW9sUntcIPquDLOnucu6LxumG-ddgFI?usp=sharing</t>
         </is>
       </c>
     </row>
@@ -815,7 +815,7 @@
       </c>
       <c r="B15" s="23" t="inlineStr">
         <is>
-          <t>submission/videos/TECHNICAL_DEMO.mp4</t>
+          <t>https://drive.google.com/drive/folders/1_zW9sUntcIPquDLOnucu6LxumG-ddgFI?usp=sharing</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>Google Gemini 3.5 Flash Lite (live API), Claude 3.5 Sonnet &amp; OpenAI GPT-4o (research benchmarking), SerpApi &amp; Google CSE (SERP integration design), Python standard library, Node.js SQLite WAL, Playwright, React 19, Tailwind CSS v4</t>
+          <t>Google Gemini 2.5 Flash, OpenAI GPT-4o / ChatGPT, Claude 3.5 Sonnet, Perplexity Sonar, Python, Node.js SQLite WAL, Playwright, React 19, Tailwind CSS v4</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>$0.00 (Zero paid tools required; free-tier APIs and standard libraries used exclusively)</t>
+          <t>$0.00 (Zero paid tools; free-tier APIs and standard libraries used exclusively)</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" style="14" min="1" max="1"/>
     <col width="24" customWidth="1" style="14" min="2" max="2"/>
@@ -1342,7 +1342,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:V304"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" style="14" min="1" max="1"/>
     <col width="40" customWidth="1" style="14" min="2" max="2"/>
@@ -1565,7 +1565,7 @@
       </c>
       <c r="G5" s="27" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>Not ranked (&gt;100)</t>
         </is>
       </c>
       <c r="H5" s="27" t="inlineStr">
@@ -4865,7 +4865,7 @@
       </c>
       <c r="G35" s="27" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>Not ranked (&gt;100)</t>
         </is>
       </c>
       <c r="H35" s="27" t="inlineStr">
@@ -8055,7 +8055,7 @@
       </c>
       <c r="G64" s="27" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>Not ranked (&gt;100)</t>
         </is>
       </c>
       <c r="H64" s="27" t="inlineStr">
@@ -18593,7 +18593,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:L54"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" style="14" min="1" max="1"/>
     <col width="30" customWidth="1" style="14" min="2" max="2"/>
@@ -20622,7 +20622,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:K84"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" style="14" min="1" max="1"/>
     <col width="14" customWidth="1" style="14" min="2" max="2"/>
@@ -20911,7 +20911,7 @@
       </c>
       <c r="D8" s="27" t="inlineStr">
         <is>
-          <t>How to Create Talking-Head Videos &amp; Podcast Narration with AI Voice Cloning and Digital Avatars</t>
+          <t>How to Create Talking-Head Videos with AI Voice Cloning &amp; Avatars</t>
         </is>
       </c>
       <c r="E8" s="27" t="inlineStr">
@@ -21141,7 +21141,7 @@
       </c>
       <c r="F12" s="27" t="inlineStr">
         <is>
-          <t>Podcasters break out of audio-only discovery bottlenecks by uploading their episode recording to an AI Creator Studio that converts audio/video into 12 vertical video clips, burned-in captions, written show notes, and LinkedIn posts. From the same screen, hosts can distribute the full episode to Spotify and YouTube while fanning out short teaser clips to Instagram, LinkedIn, and Bluesky.</t>
+          <t>Podcasters break out of audio-only discovery bottlenecks by uploading their episode recording to IncuBrix Creator Studio to automatically convert audio/video into 12 vertical video clips, burned-in captions, written show notes, and LinkedIn posts. From the same screen, hosts can distribute the full episode to Spotify and YouTube while fanning out short teaser clips to Instagram, LinkedIn, and Bluesky.</t>
         </is>
       </c>
       <c r="G12" s="27" t="inlineStr">
@@ -23721,7 +23721,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:H31"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="40" customWidth="1" style="14" min="1" max="1"/>
     <col width="14" customWidth="1" style="14" min="2" max="2"/>
@@ -24078,13 +24078,19 @@
           <t>6 merged variants</t>
         </is>
       </c>
-      <c r="F18" s="23" t="inlineStr">
-        <is>
-          <t>0.05</t>
-        </is>
-      </c>
-      <c r="G18" s="23" t="n"/>
-      <c r="H18" s="23" t="n"/>
+      <c r="F18" s="23" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G18" s="23" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="H18" s="23" t="inlineStr">
+        <is>
+          <t>logs/engine_runs.log &amp; exports/visibility.csv</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="15">
       <c r="A19" s="22" t="inlineStr">
@@ -24112,13 +24118,19 @@
           <t>0 new (idempotent)</t>
         </is>
       </c>
-      <c r="F19" s="23" t="inlineStr">
-        <is>
-          <t>0.02</t>
-        </is>
-      </c>
-      <c r="G19" s="23" t="n"/>
-      <c r="H19" s="23" t="n"/>
+      <c r="F19" s="23" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G19" s="23" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="H19" s="23" t="inlineStr">
+        <is>
+          <t>logs/engine_runs.log (identical row counts)</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="15">
       <c r="A20" s="22" t="inlineStr">
@@ -24146,13 +24158,19 @@
           <t>1 duplicate merged</t>
         </is>
       </c>
-      <c r="F20" s="23" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
-      <c r="G20" s="23" t="n"/>
-      <c r="H20" s="23" t="n"/>
+      <c r="F20" s="23" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G20" s="23" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="H20" s="23" t="inlineStr">
+        <is>
+          <t>logs/engine_runs.log (incremental upsert)</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="15">
       <c r="A21" s="22" t="inlineStr">
@@ -24180,13 +24198,19 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F21" s="23" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
-      <c r="G21" s="23" t="n"/>
-      <c r="H21" s="23" t="n"/>
+      <c r="F21" s="23" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G21" s="23" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="H21" s="23" t="inlineStr">
+        <is>
+          <t>logs/engine_runs.log (graceful retry/catch)</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="15">
       <c r="A23" s="20" t="inlineStr">
@@ -24353,8 +24377,8 @@
     <mergeCell ref="B28:H28"/>
     <mergeCell ref="B26:H26"/>
     <mergeCell ref="B27:H27"/>
+    <mergeCell ref="A16:H16"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A16:H16"/>
     <mergeCell ref="B24:H24"/>
     <mergeCell ref="B30:H30"/>
     <mergeCell ref="B29:H29"/>
@@ -24381,7 +24405,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F29"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="52" customWidth="1" style="14" min="1" max="1"/>
     <col width="14" customWidth="1" style="14" min="2" max="2"/>

</xml_diff>